<commit_message>
rework acct_profiling_vn.py script and added few more chart user breakdown
</commit_message>
<xml_diff>
--- a/data/result_20260903_142231 (user extra info).xlsx
+++ b/data/result_20260903_142231 (user extra info).xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wei.kc\Desktop\Adhoc\03 Sept 2026\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:8001_{2B29246A-9348-47EB-AE84-0C796430CE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E026FEE-7E56-48F0-88D4-AA5C3A265816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results export" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results export'!$A$1:$W$17</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="128">
   <si>
     <t>user_id</t>
   </si>
@@ -414,6 +417,9 @@
   </si>
   <si>
     <t>zpkcsnbutd@gmail.com</t>
+  </si>
+  <si>
+    <t>filter</t>
   </si>
 </sst>
 </file>
@@ -793,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:W17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
@@ -818,9 +824,10 @@
     <col min="20" max="20" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -887,8 +894,11 @@
       <c r="V1" s="1" t="s">
         <v>102</v>
       </c>
+      <c r="W1" s="1" t="s">
+        <v>127</v>
+      </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -948,7 +958,7 @@
       </c>
       <c r="T2" s="2">
         <f ca="1">INT(TODAY() - DATEVALUE(B2))</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="U2">
         <f>YEAR(B2)</f>
@@ -958,8 +968,12 @@
         <f>MONTH(B2)</f>
         <v>8</v>
       </c>
+      <c r="W2" t="str">
+        <f ca="1">IF(T2&lt;30,"&lt;30 days",IF(AND(T2&gt;=30,T2&lt;=90),"30 - 90 days","&gt;90 days"))</f>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -1019,7 +1033,7 @@
       </c>
       <c r="T3" s="2">
         <f t="shared" ref="T3:T17" ca="1" si="0">INT(TODAY() - DATEVALUE(B3))</f>
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="U3">
         <f t="shared" ref="U3:U17" si="1">YEAR(B3)</f>
@@ -1029,8 +1043,12 @@
         <f t="shared" ref="V3:V17" si="2">MONTH(B3)</f>
         <v>7</v>
       </c>
+      <c r="W3" t="str">
+        <f t="shared" ref="W3:W17" ca="1" si="3">IF(T3&lt;30,"&lt;30 days",IF(AND(T3&gt;=30,T3&lt;=90),"30 - 90 days","&gt;90 days"))</f>
+        <v>30 - 90 days</v>
+      </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1090,7 +1108,7 @@
       </c>
       <c r="T4" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="U4">
         <f t="shared" si="1"/>
@@ -1100,8 +1118,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W4" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1161,7 +1183,7 @@
       </c>
       <c r="T5" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="U5">
         <f t="shared" si="1"/>
@@ -1171,8 +1193,12 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
+      <c r="W5" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>30 - 90 days</v>
+      </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -1232,7 +1258,7 @@
       </c>
       <c r="T6" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="U6">
         <f t="shared" si="1"/>
@@ -1242,8 +1268,12 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
+      <c r="W6" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>30 - 90 days</v>
+      </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1303,7 +1333,7 @@
       </c>
       <c r="T7" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="U7">
         <f t="shared" si="1"/>
@@ -1313,8 +1343,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W7" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>30 - 90 days</v>
+      </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>49</v>
       </c>
@@ -1374,7 +1408,7 @@
       </c>
       <c r="T8" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="U8">
         <f t="shared" si="1"/>
@@ -1384,8 +1418,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W8" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>55</v>
       </c>
@@ -1445,7 +1483,7 @@
       </c>
       <c r="T9" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="U9">
         <f t="shared" si="1"/>
@@ -1455,8 +1493,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W9" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>59</v>
       </c>
@@ -1516,7 +1558,7 @@
       </c>
       <c r="T10" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="U10">
         <f t="shared" si="1"/>
@@ -1526,8 +1568,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W10" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>63</v>
       </c>
@@ -1587,7 +1633,7 @@
       </c>
       <c r="T11" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="U11">
         <f t="shared" si="1"/>
@@ -1597,8 +1643,12 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
+      <c r="W11" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>30 - 90 days</v>
+      </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>67</v>
       </c>
@@ -1658,7 +1708,7 @@
       </c>
       <c r="T12" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U12">
         <f t="shared" si="1"/>
@@ -1668,8 +1718,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W12" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>71</v>
       </c>
@@ -1729,7 +1783,7 @@
       </c>
       <c r="T13" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="U13">
         <f t="shared" si="1"/>
@@ -1739,8 +1793,12 @@
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
+      <c r="W13" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
+      </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -1800,7 +1858,7 @@
       </c>
       <c r="T14" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="U14">
         <f t="shared" si="1"/>
@@ -1810,8 +1868,12 @@
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
+      <c r="W14" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&gt;90 days</v>
+      </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>81</v>
       </c>
@@ -1871,7 +1933,7 @@
       </c>
       <c r="T15" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="U15">
         <f t="shared" si="1"/>
@@ -1881,8 +1943,12 @@
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
+      <c r="W15" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>30 - 90 days</v>
+      </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>88</v>
       </c>
@@ -1942,7 +2008,7 @@
       </c>
       <c r="T16" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>1711</v>
+        <v>1715</v>
       </c>
       <c r="U16">
         <f t="shared" si="1"/>
@@ -1952,8 +2018,12 @@
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
+      <c r="W16" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&gt;90 days</v>
+      </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>94</v>
       </c>
@@ -2013,7 +2083,7 @@
       </c>
       <c r="T17" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="U17">
         <f t="shared" si="1"/>
@@ -2022,6 +2092,10 @@
       <c r="V17">
         <f t="shared" si="2"/>
         <v>8</v>
+      </c>
+      <c r="W17" t="str">
+        <f t="shared" ca="1" si="3"/>
+        <v>&lt;30 days</v>
       </c>
     </row>
   </sheetData>

</xml_diff>